<commit_message>
Menu: the four crispy burgers, and a seed that adds missing items (A-66)
Two new categories from the updated docs/smashed_menu.xlsx, with their
pictures. The seed skipped the whole menu once any item existed, so a
server seeded at install could never have received them. It now adds
only the categories and items that are missing, and changes none that
exist: a supervisor's price stays, a hidden item stays hidden.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/smashed_menu.xlsx
+++ b/docs/smashed_menu.xlsx
@@ -84,7 +84,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -106,11 +106,55 @@
         <color rgb="00D9D9D9"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -140,6 +184,8 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -239,6 +285,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -264,6 +313,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -289,6 +341,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -314,6 +369,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -339,6 +397,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -364,6 +425,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -389,6 +453,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -414,6 +481,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -439,6 +509,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -464,6 +537,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -489,6 +565,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -514,6 +593,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -539,6 +621,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -547,7 +632,7 @@
     <from>
       <col>4</col>
       <colOff>66675</colOff>
-      <row>21</row>
+      <row>27</row>
       <rowOff>28575</rowOff>
     </from>
     <ext cx="1504950" cy="638175"/>
@@ -564,106 +649,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>4</col>
-      <colOff>66675</colOff>
-      <row>22</row>
-      <rowOff>28575</rowOff>
-    </from>
-    <ext cx="1504950" cy="590550"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="15" name="Image 15" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId15"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>4</col>
-      <colOff>66675</colOff>
-      <row>23</row>
-      <rowOff>28575</rowOff>
-    </from>
-    <ext cx="1504950" cy="561975"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="16" name="Image 16" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId16"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>4</col>
-      <colOff>200025</colOff>
-      <row>25</row>
-      <rowOff>28575</rowOff>
-    </from>
-    <ext cx="1247775" cy="819150"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="17" name="Image 17" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId17"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>4</col>
-      <colOff>352425</colOff>
-      <row>27</row>
-      <rowOff>28575</rowOff>
-    </from>
-    <ext cx="942975" cy="819150"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="18" name="Image 18" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId18"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -675,20 +663,23 @@
       <row>28</row>
       <rowOff>28575</rowOff>
     </from>
-    <ext cx="1504950" cy="704850"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="19" name="Image 19" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId19"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+    <ext cx="1504950" cy="590550"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="15" name="Image 15" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId15"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -700,20 +691,79 @@
       <row>29</row>
       <rowOff>28575</rowOff>
     </from>
-    <ext cx="1504950" cy="647700"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="20" name="Image 20" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId20"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+    <ext cx="1504950" cy="561975"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="16" name="Image 16" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId16"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>200025</colOff>
+      <row>31</row>
+      <rowOff>28575</rowOff>
+    </from>
+    <ext cx="1247775" cy="819150"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="17" name="Image 17" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId17"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>352425</colOff>
+      <row>33</row>
+      <rowOff>28575</rowOff>
+    </from>
+    <ext cx="942975" cy="819150"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="18" name="Image 18" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId18"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -722,98 +772,26 @@
     <from>
       <col>4</col>
       <colOff>66675</colOff>
-      <row>31</row>
-      <rowOff>28575</rowOff>
-    </from>
-    <ext cx="1504950" cy="790575"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="21" name="Image 21" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId21"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>4</col>
-      <colOff>190500</colOff>
-      <row>32</row>
-      <rowOff>28575</rowOff>
-    </from>
-    <ext cx="1257300" cy="819150"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="22" name="Image 22" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId22"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>4</col>
-      <colOff>66675</colOff>
-      <row>33</row>
-      <rowOff>28575</rowOff>
-    </from>
-    <ext cx="1504950" cy="657225"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="23" name="Image 23" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId23"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>4</col>
-      <colOff>133350</colOff>
       <row>34</row>
       <rowOff>28575</rowOff>
     </from>
-    <ext cx="1381125" cy="819150"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="24" name="Image 24" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId24"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+    <ext cx="1504950" cy="704850"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="19" name="Image 19" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId19"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -825,6 +803,146 @@
       <row>35</row>
       <rowOff>28575</rowOff>
     </from>
+    <ext cx="1504950" cy="647700"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="20" name="Image 20" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId20"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>66675</colOff>
+      <row>37</row>
+      <rowOff>28575</rowOff>
+    </from>
+    <ext cx="1504950" cy="790575"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="21" name="Image 21" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId21"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>190500</colOff>
+      <row>38</row>
+      <rowOff>28575</rowOff>
+    </from>
+    <ext cx="1257300" cy="819150"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="22" name="Image 22" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId22"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>66675</colOff>
+      <row>39</row>
+      <rowOff>28575</rowOff>
+    </from>
+    <ext cx="1504950" cy="657225"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="23" name="Image 23" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId23"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>133350</colOff>
+      <row>40</row>
+      <rowOff>28575</rowOff>
+    </from>
+    <ext cx="1381125" cy="819150"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="24" name="Image 24" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId24"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>66675</colOff>
+      <row>41</row>
+      <rowOff>28575</rowOff>
+    </from>
     <ext cx="1504950" cy="752475"/>
     <pic>
       <nvPicPr>
@@ -839,6 +957,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -847,7 +968,7 @@
     <from>
       <col>4</col>
       <colOff>295275</colOff>
-      <row>36</row>
+      <row>42</row>
       <rowOff>28575</rowOff>
     </from>
     <ext cx="1047750" cy="819150"/>
@@ -864,6 +985,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -872,7 +996,7 @@
     <from>
       <col>4</col>
       <colOff>152400</colOff>
-      <row>37</row>
+      <row>43</row>
       <rowOff>28575</rowOff>
     </from>
     <ext cx="1333500" cy="819150"/>
@@ -889,156 +1013,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>4</col>
-      <colOff>142875</colOff>
-      <row>39</row>
-      <rowOff>28575</rowOff>
-    </from>
-    <ext cx="1362075" cy="819150"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="28" name="Image 28" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId28"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>4</col>
-      <colOff>142875</colOff>
-      <row>40</row>
-      <rowOff>28575</rowOff>
-    </from>
-    <ext cx="1362075" cy="819150"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="29" name="Image 29" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId29"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>4</col>
-      <colOff>142875</colOff>
-      <row>41</row>
-      <rowOff>28575</rowOff>
-    </from>
-    <ext cx="1362075" cy="819150"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="30" name="Image 30" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId30"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>4</col>
-      <colOff>142875</colOff>
-      <row>42</row>
-      <rowOff>28575</rowOff>
-    </from>
-    <ext cx="1362075" cy="819150"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="31" name="Image 31" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId31"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>4</col>
-      <colOff>142875</colOff>
-      <row>43</row>
-      <rowOff>28575</rowOff>
-    </from>
-    <ext cx="1362075" cy="819150"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="32" name="Image 32" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId32"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>4</col>
-      <colOff>142875</colOff>
-      <row>44</row>
-      <rowOff>28575</rowOff>
-    </from>
-    <ext cx="1362075" cy="819150"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="33" name="Image 33" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId33"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1053,17 +1030,20 @@
     <ext cx="1362075" cy="819150"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="34" name="Image 34" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId34"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <cNvPr id="28" name="Image 28" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId28"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1078,17 +1058,20 @@
     <ext cx="1362075" cy="819150"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="35" name="Image 35" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId35"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <cNvPr id="29" name="Image 29" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId29"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1103,6 +1086,174 @@
     <ext cx="1362075" cy="819150"/>
     <pic>
       <nvPicPr>
+        <cNvPr id="30" name="Image 30" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId30"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>142875</colOff>
+      <row>48</row>
+      <rowOff>28575</rowOff>
+    </from>
+    <ext cx="1362075" cy="819150"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="31" name="Image 31" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId31"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>142875</colOff>
+      <row>49</row>
+      <rowOff>28575</rowOff>
+    </from>
+    <ext cx="1362075" cy="819150"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="32" name="Image 32" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId32"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>142875</colOff>
+      <row>50</row>
+      <rowOff>28575</rowOff>
+    </from>
+    <ext cx="1362075" cy="819150"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="33" name="Image 33" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId33"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>142875</colOff>
+      <row>51</row>
+      <rowOff>28575</rowOff>
+    </from>
+    <ext cx="1362075" cy="819150"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="34" name="Image 34" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId34"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>142875</colOff>
+      <row>52</row>
+      <rowOff>28575</rowOff>
+    </from>
+    <ext cx="1362075" cy="819150"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="35" name="Image 35" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId35"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>142875</colOff>
+      <row>53</row>
+      <rowOff>28575</rowOff>
+    </from>
+    <ext cx="1362075" cy="819150"/>
+    <pic>
+      <nvPicPr>
         <cNvPr id="36" name="Image 36" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
@@ -1114,6 +1265,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1122,7 +1276,7 @@
     <from>
       <col>4</col>
       <colOff>647700</colOff>
-      <row>49</row>
+      <row>55</row>
       <rowOff>28575</rowOff>
     </from>
     <ext cx="342900" cy="819150"/>
@@ -1139,6 +1293,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1147,7 +1304,7 @@
     <from>
       <col>4</col>
       <colOff>638175</colOff>
-      <row>50</row>
+      <row>56</row>
       <rowOff>28575</rowOff>
     </from>
     <ext cx="361950" cy="819150"/>
@@ -1164,6 +1321,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1172,7 +1332,7 @@
     <from>
       <col>4</col>
       <colOff>609600</colOff>
-      <row>51</row>
+      <row>57</row>
       <rowOff>28575</rowOff>
     </from>
     <ext cx="419100" cy="819150"/>
@@ -1189,6 +1349,121 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>133350</colOff>
+      <row>21</row>
+      <rowOff>28575</rowOff>
+    </from>
+    <ext cx="1381125" cy="657225"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="40" name="Image 40" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId40"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>133350</colOff>
+      <row>22</row>
+      <rowOff>28575</rowOff>
+    </from>
+    <ext cx="1381125" cy="685800"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="41" name="Image 41" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId41"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>133350</colOff>
+      <row>24</row>
+      <rowOff>28575</rowOff>
+    </from>
+    <ext cx="1381125" cy="657225"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="42" name="Image 42" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId42"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>133350</colOff>
+      <row>25</row>
+      <rowOff>28575</rowOff>
+    </from>
+    <ext cx="1381125" cy="657225"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="43" name="Image 43" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId43"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1485,7 +1760,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F60"/>
+  <dimension ref="A1:F66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1541,11 +1816,11 @@
           <t>CLASSIC SMASHED BURGER  |  كلاسيك سماشد برغر</t>
         </is>
       </c>
-      <c r="B3" s="4" t="n"/>
-      <c r="C3" s="4" t="n"/>
-      <c r="D3" s="4" t="n"/>
-      <c r="E3" s="4" t="n"/>
-      <c r="F3" s="4" t="n"/>
+      <c r="B3" s="11" t="n"/>
+      <c r="C3" s="11" t="n"/>
+      <c r="D3" s="11" t="n"/>
+      <c r="E3" s="11" t="n"/>
+      <c r="F3" s="12" t="n"/>
     </row>
     <row r="4" ht="70.5" customHeight="1">
       <c r="A4" s="5" t="inlineStr">
@@ -1665,11 +1940,11 @@
           <t>MUSHROOM SWISS SMASHED BURGER  |  ماشروم سويس سماشد برغر</t>
         </is>
       </c>
-      <c r="B8" s="4" t="n"/>
-      <c r="C8" s="4" t="n"/>
-      <c r="D8" s="4" t="n"/>
-      <c r="E8" s="4" t="n"/>
-      <c r="F8" s="4" t="n"/>
+      <c r="B8" s="11" t="n"/>
+      <c r="C8" s="11" t="n"/>
+      <c r="D8" s="11" t="n"/>
+      <c r="E8" s="11" t="n"/>
+      <c r="F8" s="12" t="n"/>
     </row>
     <row r="9" ht="60.75" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
@@ -1733,11 +2008,11 @@
           <t>ROYAL SMASHED BURGER  |  رويال سماشد برغر</t>
         </is>
       </c>
-      <c r="B11" s="4" t="n"/>
-      <c r="C11" s="4" t="n"/>
-      <c r="D11" s="4" t="n"/>
-      <c r="E11" s="4" t="n"/>
-      <c r="F11" s="4" t="n"/>
+      <c r="B11" s="11" t="n"/>
+      <c r="C11" s="11" t="n"/>
+      <c r="D11" s="11" t="n"/>
+      <c r="E11" s="11" t="n"/>
+      <c r="F11" s="12" t="n"/>
     </row>
     <row r="12" ht="53.25" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
@@ -1801,11 +2076,11 @@
           <t>ROAST BEEF SMASHED BURGER  |  روست بيف سماشد برغر</t>
         </is>
       </c>
-      <c r="B14" s="4" t="n"/>
-      <c r="C14" s="4" t="n"/>
-      <c r="D14" s="4" t="n"/>
-      <c r="E14" s="4" t="n"/>
-      <c r="F14" s="4" t="n"/>
+      <c r="B14" s="11" t="n"/>
+      <c r="C14" s="11" t="n"/>
+      <c r="D14" s="11" t="n"/>
+      <c r="E14" s="11" t="n"/>
+      <c r="F14" s="12" t="n"/>
     </row>
     <row r="15" ht="70.5" customHeight="1">
       <c r="A15" s="5" t="inlineStr">
@@ -1897,11 +2172,11 @@
           <t>FLAT BURGER  |  فلات برغر</t>
         </is>
       </c>
-      <c r="B18" s="4" t="n"/>
-      <c r="C18" s="4" t="n"/>
-      <c r="D18" s="4" t="n"/>
-      <c r="E18" s="4" t="n"/>
-      <c r="F18" s="4" t="n"/>
+      <c r="B18" s="11" t="n"/>
+      <c r="C18" s="11" t="n"/>
+      <c r="D18" s="11" t="n"/>
+      <c r="E18" s="11" t="n"/>
+      <c r="F18" s="12" t="n"/>
     </row>
     <row r="19" ht="61.5" customHeight="1">
       <c r="A19" s="5" t="inlineStr">
@@ -1962,424 +2237,392 @@
     <row r="21" ht="22" customHeight="1">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>KIDS MEALS  |  وجبات الأطفال</t>
-        </is>
-      </c>
-      <c r="B21" s="4" t="n"/>
-      <c r="C21" s="4" t="n"/>
-      <c r="D21" s="4" t="n"/>
-      <c r="E21" s="4" t="n"/>
-      <c r="F21" s="4" t="n"/>
-    </row>
-    <row r="22" ht="56.25" customHeight="1">
+          <t>CLASSIC CRISPY BURGER  |  برغر كلاسيك كرسبي</t>
+        </is>
+      </c>
+      <c r="B21" s="11" t="n"/>
+      <c r="C21" s="11" t="n"/>
+      <c r="D21" s="11" t="n"/>
+      <c r="E21" s="11" t="n"/>
+      <c r="F21" s="12" t="n"/>
+    </row>
+    <row r="22" ht="70.5" customHeight="1">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>Kids Smashed Burger</t>
+          <t>Single Crispy Burger</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>سماشد برغر (وجبة أطفال)</t>
+          <t>سنجل كرسبي برغر</t>
         </is>
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>100 g of beef, lettuce, tomato, cheese, special sauce, fries, juice, toy.</t>
+          <t>3-4 pieces of crispy fried chicken breast, mayonnaise, special sauce, lettuce, and cheddar cheese sauce. Meal = + fries + cola.</t>
         </is>
       </c>
       <c r="D22" s="8" t="inlineStr">
         <is>
-          <t>لحمة 100 غم، خس، بندورة، سبيشل صوص، جبنة، بطاطا، عصير، هدية.</t>
+          <t>3-4 قطع من صدر الدجاج المقلي والمقرمش، مايونيز، سبيشل صوص، خس، جبنة الشيدر السائلة. الوجبة تشمل بطاطا وكولا.</t>
         </is>
       </c>
       <c r="E22" s="7" t="n"/>
       <c r="F22" s="9" t="inlineStr">
         <is>
-          <t>25</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="52.5" customHeight="1">
+          <t>26 (sandwich)  /  36 (meal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="70.5" customHeight="1">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>Kids Crispy Burger</t>
+          <t>Double Crispy Burger</t>
         </is>
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>كرسبي برغر (وجبة أطفال)</t>
+          <t>دبل كرسبي برغر</t>
         </is>
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>Crispy chicken, lettuce, mayonnaise, cheese, fries, juice, toy.</t>
+          <t>6-7 pieces of crispy fried chicken breast, mayonnaise, special sauce, lettuce, and cheddar cheese sauce. Meal = + fries + cola.</t>
         </is>
       </c>
       <c r="D23" s="8" t="inlineStr">
         <is>
-          <t>دجاج كرسبي مقلي و مقرمش، خس، مايونيز، جبنة، بطاطا، عصير، هدية.</t>
+          <t>6-7 قطع من صدر الدجاج المقلي والمقرمش، مايونيز، سبيشل صوص، خس، جبنة الشيدر السائلة. الوجبة تشمل بطاطا وكولا.</t>
         </is>
       </c>
       <c r="E23" s="7" t="n"/>
       <c r="F23" s="9" t="inlineStr">
         <is>
-          <t>25</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="50.25" customHeight="1">
-      <c r="A24" s="5" t="inlineStr">
-        <is>
-          <t>Kids Crispy Meal</t>
-        </is>
-      </c>
-      <c r="B24" s="6" t="inlineStr">
-        <is>
-          <t>وجبة كرسبي (وجبة أطفال)</t>
-        </is>
-      </c>
-      <c r="C24" s="7" t="inlineStr">
-        <is>
-          <t>Crispy chicken, fries, juice, toy.</t>
-        </is>
-      </c>
-      <c r="D24" s="8" t="inlineStr">
-        <is>
-          <t>قطع دجاج كرسبي مقلي و مقرمش، بطاطا، عصير، هدية.</t>
-        </is>
-      </c>
-      <c r="E24" s="7" t="n"/>
-      <c r="F24" s="9" t="inlineStr">
-        <is>
-          <t>25</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="22" customHeight="1">
-      <c r="A25" s="3" t="inlineStr">
-        <is>
-          <t>MEALS  |  وجبات</t>
-        </is>
-      </c>
-      <c r="B25" s="4" t="n"/>
-      <c r="C25" s="4" t="n"/>
-      <c r="D25" s="4" t="n"/>
-      <c r="E25" s="4" t="n"/>
-      <c r="F25" s="4" t="n"/>
+          <t>30 (sandwich)  /  40 (meal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="22" customHeight="1">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>CRISPY CHICKEN BURGER  |  برغر دجاج كرسبي</t>
+        </is>
+      </c>
+      <c r="B24" s="11" t="n"/>
+      <c r="C24" s="11" t="n"/>
+      <c r="D24" s="11" t="n"/>
+      <c r="E24" s="11" t="n"/>
+      <c r="F24" s="12" t="n"/>
+    </row>
+    <row r="25" ht="70.5" customHeight="1">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Nachos Crispy Burger</t>
+        </is>
+      </c>
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t>ناشوز كرسبي برغر</t>
+        </is>
+      </c>
+      <c r="C25" s="7" t="inlineStr">
+        <is>
+          <t>3-4 pieces of crispy chicken, mayonnaise, nachos sauce, nachos chips, lettuce, and cheddar cheese sauce. Meal = + fries + cola.</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>3-4 قطع من صدر الدجاج المقلي والمقرمش، مايونيز، صوص جبنة الناشوز، خس، جبنة الشيدر السائلة. الوجبة تشمل بطاطا وكولا.</t>
+        </is>
+      </c>
+      <c r="E25" s="7" t="n"/>
+      <c r="F25" s="9" t="inlineStr">
+        <is>
+          <t>27 (sandwich)  /  37 (meal)</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="70.5" customHeight="1">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>Crispy Chicken Meal</t>
+          <t>Buffalo Crispy Burger</t>
         </is>
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>وجبة كرسبي الدجاج</t>
+          <t>بافلو كرسبي برغر</t>
         </is>
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>5 pieces of crispy chicken, fries, cola, bread.</t>
+          <t>3-4 pieces of crispy chicken, mayonnaise, spicy buffalo sauce, lettuce, and cheddar cheese sauce. Meal = + fries + cola.</t>
         </is>
       </c>
       <c r="D26" s="8" t="inlineStr">
         <is>
-          <t>5 قطع كرسبي، بطاطا، كولا، خبزة.</t>
+          <t>3-4 قطع من صدر الدجاج المقلي والمقرمش، مايونيز، صوص البافلو الحار، خس، جبنة الشيدر السائلة. الوجبة تشمل بطاطا وكولا.</t>
         </is>
       </c>
       <c r="E26" s="7" t="n"/>
       <c r="F26" s="9" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>27 (sandwich)  /  37 (meal)</t>
         </is>
       </c>
     </row>
     <row r="27" ht="22" customHeight="1">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>SPECIAL ITEMS  |  عروض خاصة</t>
-        </is>
-      </c>
-      <c r="B27" s="4" t="n"/>
-      <c r="C27" s="4" t="n"/>
-      <c r="D27" s="4" t="n"/>
-      <c r="E27" s="4" t="n"/>
-      <c r="F27" s="4" t="n"/>
-    </row>
-    <row r="28" ht="70.5" customHeight="1">
+          <t>KIDS MEALS  |  وجبات الأطفال</t>
+        </is>
+      </c>
+      <c r="B27" s="11" t="n"/>
+      <c r="C27" s="11" t="n"/>
+      <c r="D27" s="11" t="n"/>
+      <c r="E27" s="11" t="n"/>
+      <c r="F27" s="12" t="n"/>
+    </row>
+    <row r="28" ht="56.25" customHeight="1">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>2 Mini Burgers (any type)</t>
+          <t>Kids Smashed Burger</t>
         </is>
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>2 ميني برجر (أي نوع)</t>
+          <t>سماشد برغر (وجبة أطفال)</t>
         </is>
       </c>
       <c r="C28" s="7" t="inlineStr">
         <is>
-          <t>With fries, cola and sauces.</t>
+          <t>100 g of beef, lettuce, tomato, cheese, special sauce, fries, juice, toy.</t>
         </is>
       </c>
       <c r="D28" s="8" t="inlineStr">
         <is>
-          <t>مع بطاطا وكولا وصوصات.</t>
+          <t>لحمة 100 غم، خس، بندورة، سبيشل صوص، جبنة، بطاطا، عصير، هدية.</t>
         </is>
       </c>
       <c r="E28" s="7" t="n"/>
       <c r="F28" s="9" t="inlineStr">
         <is>
-          <t>43</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="61.5" customHeight="1">
+          <t>25</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="52.5" customHeight="1">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>4 Smashed Bites</t>
+          <t>Kids Crispy Burger</t>
         </is>
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>4 لقيمات سماشد</t>
+          <t>كرسبي برغر (وجبة أطفال)</t>
         </is>
       </c>
       <c r="C29" s="7" t="inlineStr">
         <is>
-          <t>With fries, cola and sauces.</t>
+          <t>Crispy chicken, lettuce, mayonnaise, cheese, fries, juice, toy.</t>
         </is>
       </c>
       <c r="D29" s="8" t="inlineStr">
         <is>
-          <t>مع بطاطا وكولا وصوصات.</t>
+          <t>دجاج كرسبي مقلي و مقرمش، خس، مايونيز، جبنة، بطاطا، عصير، هدية.</t>
         </is>
       </c>
       <c r="E29" s="7" t="n"/>
       <c r="F29" s="9" t="inlineStr">
         <is>
-          <t>40</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="57" customHeight="1">
+          <t>25</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="50.25" customHeight="1">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>Smashed Bites combo (bites + fries + cola)</t>
+          <t>Kids Crispy Meal</t>
         </is>
       </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>عرض لقيمات سماشد (لقيمات + بطاطا + كولا)</t>
+          <t>وجبة كرسبي (وجبة أطفال)</t>
         </is>
       </c>
       <c r="C30" s="7" t="inlineStr">
         <is>
-          <t>Shown in the Special Items photo, but no name or price is printed next to it.</t>
+          <t>Crispy chicken, fries, juice, toy.</t>
         </is>
       </c>
       <c r="D30" s="8" t="inlineStr">
         <is>
-          <t>ظاهر في صورة العروض الخاصة، لكن لا يوجد اسم أو سعر مكتوب بجانبه.</t>
+          <t>قطع دجاج كرسبي مقلي و مقرمش، بطاطا، عصير، هدية.</t>
         </is>
       </c>
       <c r="E30" s="7" t="n"/>
       <c r="F30" s="9" t="inlineStr">
         <is>
-          <t>not shown on menu</t>
+          <t>25</t>
         </is>
       </c>
     </row>
     <row r="31" ht="22" customHeight="1">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>APPETIZERS  |  المقبلات</t>
-        </is>
-      </c>
-      <c r="B31" s="4" t="n"/>
-      <c r="C31" s="4" t="n"/>
-      <c r="D31" s="4" t="n"/>
-      <c r="E31" s="4" t="n"/>
-      <c r="F31" s="4" t="n"/>
-    </row>
-    <row r="32" ht="68.25" customHeight="1">
+          <t>MEALS  |  وجبات</t>
+        </is>
+      </c>
+      <c r="B31" s="11" t="n"/>
+      <c r="C31" s="11" t="n"/>
+      <c r="D31" s="11" t="n"/>
+      <c r="E31" s="11" t="n"/>
+      <c r="F31" s="12" t="n"/>
+    </row>
+    <row r="32" ht="70.5" customHeight="1">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>Crispy Chicken Pieces</t>
+          <t>Crispy Chicken Meal</t>
         </is>
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>قطع كرسبي</t>
+          <t>وجبة كرسبي الدجاج</t>
         </is>
       </c>
       <c r="C32" s="7" t="inlineStr">
         <is>
-          <t>5 pieces.</t>
+          <t>5 pieces of crispy chicken, fries, cola, bread.</t>
         </is>
       </c>
       <c r="D32" s="8" t="inlineStr">
         <is>
-          <t>5 قطع.</t>
+          <t>5 قطع كرسبي، بطاطا، كولا، خبزة.</t>
         </is>
       </c>
       <c r="E32" s="7" t="n"/>
       <c r="F32" s="9" t="inlineStr">
         <is>
-          <t>25</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="70.5" customHeight="1">
-      <c r="A33" s="5" t="inlineStr">
-        <is>
-          <t>Onion Rings</t>
-        </is>
-      </c>
-      <c r="B33" s="6" t="inlineStr">
-        <is>
-          <t>حلقات البصل</t>
-        </is>
-      </c>
-      <c r="C33" s="7" t="inlineStr">
-        <is>
-          <t>5 pieces.</t>
-        </is>
-      </c>
-      <c r="D33" s="8" t="inlineStr">
-        <is>
-          <t>5 قطع.</t>
-        </is>
-      </c>
-      <c r="E33" s="7" t="n"/>
-      <c r="F33" s="9" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="57.75" customHeight="1">
+          <t>35</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="22" customHeight="1">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>SPECIAL ITEMS  |  عروض خاصة</t>
+        </is>
+      </c>
+      <c r="B33" s="11" t="n"/>
+      <c r="C33" s="11" t="n"/>
+      <c r="D33" s="11" t="n"/>
+      <c r="E33" s="11" t="n"/>
+      <c r="F33" s="12" t="n"/>
+    </row>
+    <row r="34" ht="70.5" customHeight="1">
       <c r="A34" s="5" t="inlineStr">
         <is>
-          <t>Mozzarella Sticks</t>
+          <t>2 Mini Burgers (any type)</t>
         </is>
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>اصابع موزاريلا</t>
+          <t>2 ميني برجر (أي نوع)</t>
         </is>
       </c>
       <c r="C34" s="7" t="inlineStr">
         <is>
-          <t>4 pieces.</t>
+          <t>With fries, cola and sauces.</t>
         </is>
       </c>
       <c r="D34" s="8" t="inlineStr">
         <is>
-          <t>4 قطع.</t>
+          <t>مع بطاطا وكولا وصوصات.</t>
         </is>
       </c>
       <c r="E34" s="7" t="n"/>
       <c r="F34" s="9" t="inlineStr">
         <is>
-          <t>20</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="70.5" customHeight="1">
+          <t>43</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="61.5" customHeight="1">
       <c r="A35" s="5" t="inlineStr">
         <is>
-          <t>Chicken Wings</t>
+          <t>4 Smashed Bites</t>
         </is>
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>أجنحة دجاج</t>
+          <t>4 لقيمات سماشد</t>
         </is>
       </c>
       <c r="C35" s="7" t="inlineStr">
         <is>
-          <t>10 pieces.</t>
+          <t>With fries, cola and sauces.</t>
         </is>
       </c>
       <c r="D35" s="8" t="inlineStr">
         <is>
-          <t>10 قطع.</t>
+          <t>مع بطاطا وكولا وصوصات.</t>
         </is>
       </c>
       <c r="E35" s="7" t="n"/>
       <c r="F35" s="9" t="inlineStr">
         <is>
-          <t>25</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="65.25" customHeight="1">
+          <t>40</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="57" customHeight="1">
       <c r="A36" s="5" t="inlineStr">
         <is>
-          <t>Cheese Fries Crispy</t>
+          <t>Smashed Bites combo (bites + fries + cola)</t>
         </is>
       </c>
       <c r="B36" s="6" t="inlineStr">
         <is>
-          <t>قطع كرسبي مع بطاطا بالجبنة</t>
+          <t>عرض لقيمات سماشد (لقيمات + بطاطا + كولا)</t>
         </is>
       </c>
       <c r="C36" s="7" t="inlineStr">
         <is>
-          <t>Crispy chicken pieces with cheese fries. Piece count not printed.</t>
+          <t>Shown in the Special Items photo, but no name or price is printed next to it.</t>
         </is>
       </c>
       <c r="D36" s="8" t="inlineStr">
         <is>
-          <t>قطع كرسبي مع بطاطا بالجبنة. عدد القطع غير مذكور.</t>
+          <t>ظاهر في صورة العروض الخاصة، لكن لا يوجد اسم أو سعر مكتوب بجانبه.</t>
         </is>
       </c>
       <c r="E36" s="7" t="n"/>
       <c r="F36" s="9" t="inlineStr">
         <is>
-          <t>25</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="70.5" customHeight="1">
-      <c r="A37" s="5" t="inlineStr">
-        <is>
-          <t>Chicken Pop Corn</t>
-        </is>
-      </c>
-      <c r="B37" s="6" t="inlineStr">
-        <is>
-          <t>تشكن بوب كورن</t>
-        </is>
-      </c>
-      <c r="C37" s="7" t="inlineStr">
-        <is>
-          <t>12 pieces.</t>
-        </is>
-      </c>
-      <c r="D37" s="8" t="inlineStr">
-        <is>
-          <t>12 قطعة.</t>
-        </is>
-      </c>
-      <c r="E37" s="7" t="n"/>
-      <c r="F37" s="9" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="70.5" customHeight="1">
+          <t>not shown on menu</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="22" customHeight="1">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>APPETIZERS  |  المقبلات</t>
+        </is>
+      </c>
+      <c r="B37" s="11" t="n"/>
+      <c r="C37" s="11" t="n"/>
+      <c r="D37" s="11" t="n"/>
+      <c r="E37" s="11" t="n"/>
+      <c r="F37" s="12" t="n"/>
+    </row>
+    <row r="38" ht="68.25" customHeight="1">
       <c r="A38" s="5" t="inlineStr">
         <is>
-          <t>Jalapeño Cheddar Bites</t>
+          <t>Crispy Chicken Pieces</t>
         </is>
       </c>
       <c r="B38" s="6" t="inlineStr">
         <is>
-          <t>كرات الجبنة مع الهالبينو</t>
+          <t>قطع كرسبي</t>
         </is>
       </c>
       <c r="C38" s="7" t="inlineStr">
@@ -2395,546 +2638,716 @@
       <c r="E38" s="7" t="n"/>
       <c r="F38" s="9" t="inlineStr">
         <is>
-          <t>15</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="22" customHeight="1">
-      <c r="A39" s="3" t="inlineStr">
-        <is>
-          <t>FRIES  |  بطاطا</t>
-        </is>
-      </c>
-      <c r="B39" s="4" t="n"/>
-      <c r="C39" s="4" t="n"/>
-      <c r="D39" s="4" t="n"/>
-      <c r="E39" s="4" t="n"/>
-      <c r="F39" s="4" t="n"/>
-    </row>
-    <row r="40" ht="70.5" customHeight="1">
+          <t>25</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="70.5" customHeight="1">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>Onion Rings</t>
+        </is>
+      </c>
+      <c r="B39" s="6" t="inlineStr">
+        <is>
+          <t>حلقات البصل</t>
+        </is>
+      </c>
+      <c r="C39" s="7" t="inlineStr">
+        <is>
+          <t>5 pieces.</t>
+        </is>
+      </c>
+      <c r="D39" s="8" t="inlineStr">
+        <is>
+          <t>5 قطع.</t>
+        </is>
+      </c>
+      <c r="E39" s="7" t="n"/>
+      <c r="F39" s="9" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="57.75" customHeight="1">
       <c r="A40" s="5" t="inlineStr">
         <is>
-          <t>French Fries (S)</t>
+          <t>Mozzarella Sticks</t>
         </is>
       </c>
       <c r="B40" s="6" t="inlineStr">
         <is>
-          <t>بطاطا عادية (صغير)</t>
+          <t>اصابع موزاريلا</t>
         </is>
       </c>
       <c r="C40" s="7" t="inlineStr">
         <is>
-          <t>Straight-cut fries, small.</t>
+          <t>4 pieces.</t>
         </is>
       </c>
       <c r="D40" s="8" t="inlineStr">
         <is>
-          <t>بطاطا عادية، حجم صغير.</t>
+          <t>4 قطع.</t>
         </is>
       </c>
       <c r="E40" s="7" t="n"/>
       <c r="F40" s="9" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>20</t>
         </is>
       </c>
     </row>
     <row r="41" ht="70.5" customHeight="1">
       <c r="A41" s="5" t="inlineStr">
         <is>
-          <t>French Fries (L)</t>
+          <t>Chicken Wings</t>
         </is>
       </c>
       <c r="B41" s="6" t="inlineStr">
         <is>
-          <t>بطاطا عادية (كبير)</t>
+          <t>أجنحة دجاج</t>
         </is>
       </c>
       <c r="C41" s="7" t="inlineStr">
         <is>
-          <t>Straight-cut fries, large.</t>
+          <t>10 pieces.</t>
         </is>
       </c>
       <c r="D41" s="8" t="inlineStr">
         <is>
-          <t>بطاطا عادية، حجم كبير.</t>
+          <t>10 قطع.</t>
         </is>
       </c>
       <c r="E41" s="7" t="n"/>
       <c r="F41" s="9" t="inlineStr">
         <is>
-          <t>16</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="70.5" customHeight="1">
+          <t>25</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="65.25" customHeight="1">
       <c r="A42" s="5" t="inlineStr">
         <is>
-          <t>Cheese French Fries Jalapeño</t>
+          <t>Cheese Fries Crispy</t>
         </is>
       </c>
       <c r="B42" s="6" t="inlineStr">
         <is>
-          <t>بطاطا عادية مع جبنة وهالبينو</t>
+          <t>قطع كرسبي مع بطاطا بالجبنة</t>
         </is>
       </c>
       <c r="C42" s="7" t="inlineStr">
         <is>
-          <t>Straight-cut fries with cheese and jalapeño.</t>
+          <t>Crispy chicken pieces with cheese fries. Piece count not printed.</t>
         </is>
       </c>
       <c r="D42" s="8" t="inlineStr">
         <is>
-          <t>بطاطا عادية مع جبنة وهالبينو.</t>
+          <t>قطع كرسبي مع بطاطا بالجبنة. عدد القطع غير مذكور.</t>
         </is>
       </c>
       <c r="E42" s="7" t="n"/>
       <c r="F42" s="9" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>25</t>
         </is>
       </c>
     </row>
     <row r="43" ht="70.5" customHeight="1">
       <c r="A43" s="5" t="inlineStr">
         <is>
-          <t>Curly Fries (S)</t>
+          <t>Chicken Pop Corn</t>
         </is>
       </c>
       <c r="B43" s="6" t="inlineStr">
         <is>
-          <t>بطاطا كيرلي (صغير)</t>
+          <t>تشكن بوب كورن</t>
         </is>
       </c>
       <c r="C43" s="7" t="inlineStr">
         <is>
-          <t>Curly fries, small.</t>
+          <t>12 pieces.</t>
         </is>
       </c>
       <c r="D43" s="8" t="inlineStr">
         <is>
-          <t>بطاطا كيرلي، حجم صغير.</t>
+          <t>12 قطعة.</t>
         </is>
       </c>
       <c r="E43" s="7" t="n"/>
       <c r="F43" s="9" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>20</t>
         </is>
       </c>
     </row>
     <row r="44" ht="70.5" customHeight="1">
       <c r="A44" s="5" t="inlineStr">
         <is>
-          <t>Curly Fries (L)</t>
+          <t>Jalapeño Cheddar Bites</t>
         </is>
       </c>
       <c r="B44" s="6" t="inlineStr">
         <is>
-          <t>بطاطا كيرلي (كبير)</t>
+          <t>كرات الجبنة مع الهالبينو</t>
         </is>
       </c>
       <c r="C44" s="7" t="inlineStr">
         <is>
-          <t>Curly fries, large.</t>
+          <t>5 pieces.</t>
         </is>
       </c>
       <c r="D44" s="8" t="inlineStr">
         <is>
-          <t>بطاطا كيرلي، حجم كبير.</t>
+          <t>5 قطع.</t>
         </is>
       </c>
       <c r="E44" s="7" t="n"/>
       <c r="F44" s="9" t="inlineStr">
         <is>
-          <t>20</t>
-        </is>
-      </c>
-    </row>
-    <row r="45" ht="70.5" customHeight="1">
-      <c r="A45" s="5" t="inlineStr">
-        <is>
-          <t>Cheese Curly Fries Jalapeño</t>
-        </is>
-      </c>
-      <c r="B45" s="6" t="inlineStr">
-        <is>
-          <t>بطاطا كيرلي مع جبنة وهالبينو</t>
-        </is>
-      </c>
-      <c r="C45" s="7" t="inlineStr">
-        <is>
-          <t>Curly fries with cheese and jalapeño.</t>
-        </is>
-      </c>
-      <c r="D45" s="8" t="inlineStr">
-        <is>
-          <t>بطاطا كيرلي مع جبنة وهالبينو.</t>
-        </is>
-      </c>
-      <c r="E45" s="7" t="n"/>
-      <c r="F45" s="9" t="inlineStr">
-        <is>
-          <t>25</t>
-        </is>
-      </c>
+          <t>15</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="22" customHeight="1">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>FRIES  |  بطاطا</t>
+        </is>
+      </c>
+      <c r="B45" s="11" t="n"/>
+      <c r="C45" s="11" t="n"/>
+      <c r="D45" s="11" t="n"/>
+      <c r="E45" s="11" t="n"/>
+      <c r="F45" s="12" t="n"/>
     </row>
     <row r="46" ht="70.5" customHeight="1">
       <c r="A46" s="5" t="inlineStr">
         <is>
-          <t>Wedges Fries (S)</t>
+          <t>French Fries (S)</t>
         </is>
       </c>
       <c r="B46" s="6" t="inlineStr">
         <is>
-          <t>بطاطا ويدجز (صغير)</t>
+          <t>بطاطا عادية (صغير)</t>
         </is>
       </c>
       <c r="C46" s="7" t="inlineStr">
         <is>
-          <t>Potato wedges, small.</t>
+          <t>Straight-cut fries, small.</t>
         </is>
       </c>
       <c r="D46" s="8" t="inlineStr">
         <is>
-          <t>بطاطا ويدجز، حجم صغير.</t>
+          <t>بطاطا عادية، حجم صغير.</t>
         </is>
       </c>
       <c r="E46" s="7" t="n"/>
       <c r="F46" s="9" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
     </row>
     <row r="47" ht="70.5" customHeight="1">
       <c r="A47" s="5" t="inlineStr">
         <is>
-          <t>Wedges Fries (L)</t>
+          <t>French Fries (L)</t>
         </is>
       </c>
       <c r="B47" s="6" t="inlineStr">
         <is>
-          <t>بطاطا ويدجز (كبير)</t>
+          <t>بطاطا عادية (كبير)</t>
         </is>
       </c>
       <c r="C47" s="7" t="inlineStr">
         <is>
-          <t>Potato wedges, large.</t>
+          <t>Straight-cut fries, large.</t>
         </is>
       </c>
       <c r="D47" s="8" t="inlineStr">
         <is>
-          <t>بطاطا ويدجز، حجم كبير.</t>
+          <t>بطاطا عادية، حجم كبير.</t>
         </is>
       </c>
       <c r="E47" s="7" t="n"/>
       <c r="F47" s="9" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>16</t>
         </is>
       </c>
     </row>
     <row r="48" ht="70.5" customHeight="1">
       <c r="A48" s="5" t="inlineStr">
         <is>
-          <t>Cheese Wedges Fries Jalapeño</t>
+          <t>Cheese French Fries Jalapeño</t>
         </is>
       </c>
       <c r="B48" s="6" t="inlineStr">
         <is>
-          <t>بطاطا ويدجز مع جبنة وهالبينو</t>
+          <t>بطاطا عادية مع جبنة وهالبينو</t>
         </is>
       </c>
       <c r="C48" s="7" t="inlineStr">
         <is>
-          <t>Potato wedges with cheese and jalapeño.</t>
+          <t>Straight-cut fries with cheese and jalapeño.</t>
         </is>
       </c>
       <c r="D48" s="8" t="inlineStr">
         <is>
-          <t>بطاطا ويدجز مع جبنة وهالبينو.</t>
+          <t>بطاطا عادية مع جبنة وهالبينو.</t>
         </is>
       </c>
       <c r="E48" s="7" t="n"/>
       <c r="F48" s="9" t="inlineStr">
         <is>
-          <t>25</t>
-        </is>
-      </c>
-    </row>
-    <row r="49" ht="22" customHeight="1">
-      <c r="A49" s="3" t="inlineStr">
-        <is>
-          <t>DRINKS  |  مشروبات</t>
-        </is>
-      </c>
-      <c r="B49" s="4" t="n"/>
-      <c r="C49" s="4" t="n"/>
-      <c r="D49" s="4" t="n"/>
-      <c r="E49" s="4" t="n"/>
-      <c r="F49" s="4" t="n"/>
+          <t>18</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="70.5" customHeight="1">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>Curly Fries (S)</t>
+        </is>
+      </c>
+      <c r="B49" s="6" t="inlineStr">
+        <is>
+          <t>بطاطا كيرلي (صغير)</t>
+        </is>
+      </c>
+      <c r="C49" s="7" t="inlineStr">
+        <is>
+          <t>Curly fries, small.</t>
+        </is>
+      </c>
+      <c r="D49" s="8" t="inlineStr">
+        <is>
+          <t>بطاطا كيرلي، حجم صغير.</t>
+        </is>
+      </c>
+      <c r="E49" s="7" t="n"/>
+      <c r="F49" s="9" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="70.5" customHeight="1">
       <c r="A50" s="5" t="inlineStr">
         <is>
-          <t>Water</t>
+          <t>Curly Fries (L)</t>
         </is>
       </c>
       <c r="B50" s="6" t="inlineStr">
         <is>
-          <t>ماء</t>
+          <t>بطاطا كيرلي (كبير)</t>
         </is>
       </c>
       <c r="C50" s="7" t="inlineStr">
         <is>
-          <t>Bottled water.</t>
+          <t>Curly fries, large.</t>
         </is>
       </c>
       <c r="D50" s="8" t="inlineStr">
         <is>
-          <t>مياه معبأة.</t>
+          <t>بطاطا كيرلي، حجم كبير.</t>
         </is>
       </c>
       <c r="E50" s="7" t="n"/>
       <c r="F50" s="9" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>20</t>
         </is>
       </c>
     </row>
     <row r="51" ht="70.5" customHeight="1">
       <c r="A51" s="5" t="inlineStr">
         <is>
-          <t>Juice</t>
+          <t>Cheese Curly Fries Jalapeño</t>
         </is>
       </c>
       <c r="B51" s="6" t="inlineStr">
         <is>
-          <t>عصير</t>
+          <t>بطاطا كيرلي مع جبنة وهالبينو</t>
         </is>
       </c>
       <c r="C51" s="7" t="inlineStr">
         <is>
-          <t>Bottled juice.</t>
+          <t>Curly fries with cheese and jalapeño.</t>
         </is>
       </c>
       <c r="D51" s="8" t="inlineStr">
         <is>
-          <t>عصير معبأ.</t>
+          <t>بطاطا كيرلي مع جبنة وهالبينو.</t>
         </is>
       </c>
       <c r="E51" s="7" t="n"/>
       <c r="F51" s="9" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>25</t>
         </is>
       </c>
     </row>
     <row r="52" ht="70.5" customHeight="1">
       <c r="A52" s="5" t="inlineStr">
         <is>
-          <t>Chat Cola</t>
+          <t>Wedges Fries (S)</t>
         </is>
       </c>
       <c r="B52" s="6" t="inlineStr">
         <is>
-          <t>شات كولا</t>
+          <t>بطاطا ويدجز (صغير)</t>
         </is>
       </c>
       <c r="C52" s="7" t="inlineStr">
         <is>
-          <t>Canned cola.</t>
+          <t>Potato wedges, small.</t>
         </is>
       </c>
       <c r="D52" s="8" t="inlineStr">
         <is>
-          <t>كولا علبة.</t>
+          <t>بطاطا ويدجز، حجم صغير.</t>
         </is>
       </c>
       <c r="E52" s="7" t="n"/>
       <c r="F52" s="9" t="inlineStr">
         <is>
-          <t>3</t>
-        </is>
-      </c>
-    </row>
-    <row r="53" ht="22" customHeight="1">
-      <c r="A53" s="3" t="inlineStr">
-        <is>
-          <t>ADD-ONS  |  إضافات</t>
-        </is>
-      </c>
-      <c r="B53" s="4" t="n"/>
-      <c r="C53" s="4" t="n"/>
-      <c r="D53" s="4" t="n"/>
-      <c r="E53" s="4" t="n"/>
-      <c r="F53" s="4" t="n"/>
-    </row>
-    <row r="54" ht="20" customHeight="1">
+          <t>10</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="70.5" customHeight="1">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>Wedges Fries (L)</t>
+        </is>
+      </c>
+      <c r="B53" s="6" t="inlineStr">
+        <is>
+          <t>بطاطا ويدجز (كبير)</t>
+        </is>
+      </c>
+      <c r="C53" s="7" t="inlineStr">
+        <is>
+          <t>Potato wedges, large.</t>
+        </is>
+      </c>
+      <c r="D53" s="8" t="inlineStr">
+        <is>
+          <t>بطاطا ويدجز، حجم كبير.</t>
+        </is>
+      </c>
+      <c r="E53" s="7" t="n"/>
+      <c r="F53" s="9" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="70.5" customHeight="1">
       <c r="A54" s="5" t="inlineStr">
         <is>
-          <t>Add cheese on burger</t>
+          <t>Cheese Wedges Fries Jalapeño</t>
         </is>
       </c>
       <c r="B54" s="6" t="inlineStr">
         <is>
-          <t>إضافة الجبنة على البرجر</t>
+          <t>بطاطا ويدجز مع جبنة وهالبينو</t>
         </is>
       </c>
       <c r="C54" s="7" t="inlineStr">
         <is>
-          <t>Extra cheese on any burger.</t>
+          <t>Potato wedges with cheese and jalapeño.</t>
         </is>
       </c>
       <c r="D54" s="8" t="inlineStr">
         <is>
-          <t>جبنة إضافية على أي برجر.</t>
+          <t>بطاطا ويدجز مع جبنة وهالبينو.</t>
         </is>
       </c>
       <c r="E54" s="7" t="n"/>
       <c r="F54" s="9" t="inlineStr">
         <is>
-          <t>+2</t>
-        </is>
-      </c>
-    </row>
-    <row r="55" ht="20" customHeight="1">
-      <c r="A55" s="5" t="inlineStr">
-        <is>
-          <t>Switch to curly fries</t>
-        </is>
-      </c>
-      <c r="B55" s="6" t="inlineStr">
-        <is>
-          <t>تبديل إلى كيرلي</t>
-        </is>
-      </c>
-      <c r="C55" s="7" t="inlineStr">
-        <is>
-          <t>Upgrade the meal fries to curly fries.</t>
-        </is>
-      </c>
-      <c r="D55" s="8" t="inlineStr">
-        <is>
-          <t>تبديل بطاطا الوجبة إلى كيرلي.</t>
-        </is>
-      </c>
-      <c r="E55" s="7" t="n"/>
-      <c r="F55" s="9" t="inlineStr">
-        <is>
-          <t>+4</t>
-        </is>
-      </c>
-    </row>
-    <row r="56" ht="20" customHeight="1">
+          <t>25</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="22" customHeight="1">
+      <c r="A55" s="3" t="inlineStr">
+        <is>
+          <t>DRINKS  |  مشروبات</t>
+        </is>
+      </c>
+      <c r="B55" s="11" t="n"/>
+      <c r="C55" s="11" t="n"/>
+      <c r="D55" s="11" t="n"/>
+      <c r="E55" s="11" t="n"/>
+      <c r="F55" s="12" t="n"/>
+    </row>
+    <row r="56" ht="70.5" customHeight="1">
       <c r="A56" s="5" t="inlineStr">
         <is>
-          <t>Switch to wedges fries</t>
+          <t>Water</t>
         </is>
       </c>
       <c r="B56" s="6" t="inlineStr">
         <is>
-          <t>تبديل إلى ويدجز</t>
+          <t>ماء</t>
         </is>
       </c>
       <c r="C56" s="7" t="inlineStr">
         <is>
-          <t>Upgrade the meal fries to wedges.</t>
+          <t>Bottled water.</t>
         </is>
       </c>
       <c r="D56" s="8" t="inlineStr">
         <is>
-          <t>تبديل بطاطا الوجبة إلى ويدجز.</t>
+          <t>مياه معبأة.</t>
         </is>
       </c>
       <c r="E56" s="7" t="n"/>
       <c r="F56" s="9" t="inlineStr">
         <is>
-          <t>+2</t>
-        </is>
-      </c>
-    </row>
-    <row r="57" ht="20" customHeight="1">
+          <t>3</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="70.5" customHeight="1">
       <c r="A57" s="5" t="inlineStr">
         <is>
-          <t>Add cheddar cheese sauce</t>
+          <t>Juice</t>
         </is>
       </c>
       <c r="B57" s="6" t="inlineStr">
         <is>
-          <t>إضافة صلصة جبنة شيدر سائلة</t>
+          <t>عصير</t>
         </is>
       </c>
       <c r="C57" s="7" t="inlineStr">
         <is>
-          <t>Extra cheddar cheese sauce.</t>
+          <t>Bottled juice.</t>
         </is>
       </c>
       <c r="D57" s="8" t="inlineStr">
         <is>
-          <t>صلصة جبنة شيدر سائلة إضافية.</t>
+          <t>عصير معبأ.</t>
         </is>
       </c>
       <c r="E57" s="7" t="n"/>
       <c r="F57" s="9" t="inlineStr">
         <is>
-          <t>+3</t>
-        </is>
-      </c>
-    </row>
-    <row r="58" ht="20" customHeight="1">
+          <t>3</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="70.5" customHeight="1">
       <c r="A58" s="5" t="inlineStr">
         <is>
-          <t>Add jalapeño</t>
+          <t>Chat Cola</t>
         </is>
       </c>
       <c r="B58" s="6" t="inlineStr">
         <is>
-          <t>إضافة هالبينو</t>
+          <t>شات كولا</t>
         </is>
       </c>
       <c r="C58" s="7" t="inlineStr">
         <is>
-          <t>Extra jalapeño.</t>
+          <t>Canned cola.</t>
         </is>
       </c>
       <c r="D58" s="8" t="inlineStr">
         <is>
-          <t>هالبينو إضافي.</t>
+          <t>كولا علبة.</t>
         </is>
       </c>
       <c r="E58" s="7" t="n"/>
       <c r="F58" s="9" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="22" customHeight="1">
+      <c r="A59" s="3" t="inlineStr">
+        <is>
+          <t>ADD-ONS  |  إضافات</t>
+        </is>
+      </c>
+      <c r="B59" s="11" t="n"/>
+      <c r="C59" s="11" t="n"/>
+      <c r="D59" s="11" t="n"/>
+      <c r="E59" s="11" t="n"/>
+      <c r="F59" s="12" t="n"/>
+    </row>
+    <row r="60" ht="20" customHeight="1">
+      <c r="A60" s="5" t="inlineStr">
+        <is>
+          <t>Add cheese on burger</t>
+        </is>
+      </c>
+      <c r="B60" s="6" t="inlineStr">
+        <is>
+          <t>إضافة الجبنة على البرجر</t>
+        </is>
+      </c>
+      <c r="C60" s="7" t="inlineStr">
+        <is>
+          <t>Extra cheese on any burger.</t>
+        </is>
+      </c>
+      <c r="D60" s="8" t="inlineStr">
+        <is>
+          <t>جبنة إضافية على أي برجر.</t>
+        </is>
+      </c>
+      <c r="E60" s="7" t="n"/>
+      <c r="F60" s="9" t="inlineStr">
+        <is>
+          <t>+2</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="20" customHeight="1">
+      <c r="A61" s="5" t="inlineStr">
+        <is>
+          <t>Switch to curly fries</t>
+        </is>
+      </c>
+      <c r="B61" s="6" t="inlineStr">
+        <is>
+          <t>تبديل إلى كيرلي</t>
+        </is>
+      </c>
+      <c r="C61" s="7" t="inlineStr">
+        <is>
+          <t>Upgrade the meal fries to curly fries.</t>
+        </is>
+      </c>
+      <c r="D61" s="8" t="inlineStr">
+        <is>
+          <t>تبديل بطاطا الوجبة إلى كيرلي.</t>
+        </is>
+      </c>
+      <c r="E61" s="7" t="n"/>
+      <c r="F61" s="9" t="inlineStr">
+        <is>
+          <t>+4</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="20" customHeight="1">
+      <c r="A62" s="5" t="inlineStr">
+        <is>
+          <t>Switch to wedges fries</t>
+        </is>
+      </c>
+      <c r="B62" s="6" t="inlineStr">
+        <is>
+          <t>تبديل إلى ويدجز</t>
+        </is>
+      </c>
+      <c r="C62" s="7" t="inlineStr">
+        <is>
+          <t>Upgrade the meal fries to wedges.</t>
+        </is>
+      </c>
+      <c r="D62" s="8" t="inlineStr">
+        <is>
+          <t>تبديل بطاطا الوجبة إلى ويدجز.</t>
+        </is>
+      </c>
+      <c r="E62" s="7" t="n"/>
+      <c r="F62" s="9" t="inlineStr">
+        <is>
+          <t>+2</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="20" customHeight="1">
+      <c r="A63" s="5" t="inlineStr">
+        <is>
+          <t>Add cheddar cheese sauce</t>
+        </is>
+      </c>
+      <c r="B63" s="6" t="inlineStr">
+        <is>
+          <t>إضافة صلصة جبنة شيدر سائلة</t>
+        </is>
+      </c>
+      <c r="C63" s="7" t="inlineStr">
+        <is>
+          <t>Extra cheddar cheese sauce.</t>
+        </is>
+      </c>
+      <c r="D63" s="8" t="inlineStr">
+        <is>
+          <t>صلصة جبنة شيدر سائلة إضافية.</t>
+        </is>
+      </c>
+      <c r="E63" s="7" t="n"/>
+      <c r="F63" s="9" t="inlineStr">
+        <is>
+          <t>+3</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="20" customHeight="1">
+      <c r="A64" s="5" t="inlineStr">
+        <is>
+          <t>Add jalapeño</t>
+        </is>
+      </c>
+      <c r="B64" s="6" t="inlineStr">
+        <is>
+          <t>إضافة هالبينو</t>
+        </is>
+      </c>
+      <c r="C64" s="7" t="inlineStr">
+        <is>
+          <t>Extra jalapeño.</t>
+        </is>
+      </c>
+      <c r="D64" s="8" t="inlineStr">
+        <is>
+          <t>هالبينو إضافي.</t>
+        </is>
+      </c>
+      <c r="E64" s="7" t="n"/>
+      <c r="F64" s="9" t="inlineStr">
+        <is>
           <t>FREE</t>
         </is>
       </c>
     </row>
-    <row r="60" ht="44" customHeight="1">
-      <c r="A60" s="10" t="inlineStr">
-        <is>
-          <t>Source: transcribed from the 7 Smashed menu images provided (menue-1 … menue-7.jpg); every picture is cropped from those same images. Prices in NIS (شيكل). Burgers show sandwich price / meal price — the meal adds fries and a drink. Where the menu prints only one language (fries, drinks, part of the special items), the other column is a translation, not printed text. Where the menu prints no contents or no price, the cell says so instead of guessing.</t>
+    <row r="66" ht="44" customHeight="1">
+      <c r="A66" s="10" t="inlineStr">
+        <is>
+          <t>Source: transcribed from the 8 Smashed menu images provided (menue-1 … menue-7.jpg plus the Crispy Burger page); every picture is cropped from those same images. Prices in NIS (شيكل). Burgers show sandwich price / meal price — the meal adds fries and a drink. Where the menu prints only one language (fries, drinks, part of the special items), the other column is a translation, not printed text. Where the menu prints no contents or no price, the cell says so instead of guessing.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A2:F58"/>
-  <mergeCells count="14">
+  <mergeCells count="16">
+    <mergeCell ref="A24:F24"/>
+    <mergeCell ref="A33:F33"/>
     <mergeCell ref="A11:F11"/>
-    <mergeCell ref="A49:F49"/>
-    <mergeCell ref="A60:F60"/>
     <mergeCell ref="A14:F14"/>
+    <mergeCell ref="A66:F66"/>
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A37:F37"/>
+    <mergeCell ref="A45:F45"/>
     <mergeCell ref="A27:F27"/>
+    <mergeCell ref="A31:F31"/>
     <mergeCell ref="A8:F8"/>
-    <mergeCell ref="A31:F31"/>
     <mergeCell ref="A18:F18"/>
     <mergeCell ref="A3:F3"/>
     <mergeCell ref="A21:F21"/>
-    <mergeCell ref="A39:F39"/>
-    <mergeCell ref="A53:F53"/>
-    <mergeCell ref="A25:F25"/>
+    <mergeCell ref="A55:F55"/>
+    <mergeCell ref="A59:F59"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>